<commit_message>
Junior IT Jobs - 148 jobs (15:35)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
+++ b/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK138"/>
+  <dimension ref="A1:AK149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21732,6 +21732,1935 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>J-00138</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Datenschutzerklärung</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Datenschutzerklärung</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>html, javascript</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>Impressum
+Betterbits GmbH
+Bunsenstraße 22
+64293 Darmstadt
+Kontakt:
+Tel. +49 6151-88 00 5-00
+Fax +49 6151-88 00 5-59
+Email: info@betterbits.de
+Web: betterbits.de
+Sitz der Gesellschaft: Darmstadt
+Registergericht: Amtsgericht Darmstadt HRB 99302
+Umsatzsteuer-Identifikationsnummer: DE 266392983
+Geschäftsführer: Björn Bopp
+Verantwortlich nach § 6 Abs.2 MDStV:
+Björn Bopp,
+Betterbits GmbH
+Bunsenstr. 22
+64293 Darmstadt
+Wir widersprechen der Nutzung unserer Daten zu Marketingzwecken und weisen darau</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betterbits.de/impressum</t>
+        </is>
+      </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>Bits4Soft - Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>bits4softsoftwareentwicklung</t>
+        </is>
+      </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N139" s="2" t="n"/>
+      <c r="O139" s="2" t="inlineStr">
+        <is>
+          <t>Hauptstraße 59</t>
+        </is>
+      </c>
+      <c r="P139" s="2" t="inlineStr">
+        <is>
+          <t>+49 160 6543202</t>
+        </is>
+      </c>
+      <c r="Q139" s="2" t="n"/>
+      <c r="R139" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S139" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betterbits.de/jobs</t>
+        </is>
+      </c>
+      <c r="U139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betterbits.de</t>
+        </is>
+      </c>
+      <c r="V139" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Bits4Soft - Softwareentwicklung_career.html</t>
+        </is>
+      </c>
+      <c r="W139" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Bits4Soft - Softwareentwicklung_Datenschutzerklärung.html</t>
+        </is>
+      </c>
+      <c r="X139" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y139" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z139" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA139" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB139" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="AC139" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD139" s="2" t="inlineStr"/>
+      <c r="AE139" s="2" t="inlineStr"/>
+      <c r="AF139" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:34:48</t>
+        </is>
+      </c>
+      <c r="AG139" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH139" s="2" t="n">
+        <v>2331</v>
+      </c>
+      <c r="AI139" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ139" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:34:48</t>
+        </is>
+      </c>
+      <c r="AK139" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:34:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>J-00139</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>impressum and data protection</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>impressum and data protection</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>go</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>Impressum
+Angaben gemäß § 5 TMG
+ISC International Software Consultants GmbH
+Dreieichstr. 42
+60594 Frankfurt
+Handelsregister: 47763
+Registergericht: Frankfurt am Main
+Vertreten durch: Christoph Oswald
+Telefon: +49 69 380 979 168 0
+E-Mail: ISC@intlsc.de
+Umsatzsteuer-ID
+Umsatzsteuer-Identifikationsnummer gemäß § 27 a Umsatzsteuergesetz:
+DE202753462
+Verbraucherstreitbeilegung/Universalschlichtungsstelle
+Wir nehmen an einem Streitbeilegungsverfahren vor einer Verbraucherschlichtungsst</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>https://intlsc.de/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>ISC it &amp; software consultants GmbH</t>
+        </is>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>iscitsoftwareconsultants</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N140" s="2" t="n"/>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>Wörnitzstraße 115a</t>
+        </is>
+      </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 9367576</t>
+        </is>
+      </c>
+      <c r="Q140" s="2" t="n"/>
+      <c r="R140" s="2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="S140" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T140" s="2" t="inlineStr">
+        <is>
+          <t>https://intlsc.de/</t>
+        </is>
+      </c>
+      <c r="U140" s="2" t="inlineStr">
+        <is>
+          <t>https://intlsc.de</t>
+        </is>
+      </c>
+      <c r="V140" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/ISC it _ software consultants GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="W140" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/ISC it _ software consultants GmbH_impressum and data protection.html</t>
+        </is>
+      </c>
+      <c r="X140" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y140" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z140" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA140" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB140" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="AC140" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AD140" s="2" t="inlineStr"/>
+      <c r="AE140" s="2" t="inlineStr"/>
+      <c r="AF140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:34:59</t>
+        </is>
+      </c>
+      <c r="AG140" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH140" s="2" t="n">
+        <v>2350</v>
+      </c>
+      <c r="AI140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:34:59</t>
+        </is>
+      </c>
+      <c r="AK140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:34:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>J-00140</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Initiativbewerbung Studenten (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Initiativbewerbung Studenten (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>IT-Ausbildung &amp; Studium</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr"/>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>SOFTWARE by e.solutions
+WIR bei e.solutions
+DU bei e.solutions
+KONTAKT
+Initiativbewerbung Studenten (m/w/d)
+Studierende Erlangen / Ingolstadt oa7a7zj5
+JETZT ONLINE BEWERBEN
+Die Zukunft des Autos findet im Innenraum statt. Die Software dazu entwickeln wir! Als Joint Venture der CARIAD SE und der Elektrobit Automotive GmbH entwickeln wir hochkomplexe Lösungen für die Kommunikation im und aus dem Auto. Für unsere Kunden aus dem VW-Konzern gestalten wir Frameworks, Applikationen und graphische Be</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs/details/initiativbewerbung-studenten-mwd</t>
+        </is>
+      </c>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N141" s="2" t="n"/>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P141" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q141" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R141" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S141" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V141" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W141" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/endobit software solutions_Initiativbewerbung Studenten _m_w_d.html</t>
+        </is>
+      </c>
+      <c r="X141" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y141" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z141" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA141" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB141" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="AC141" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD141" s="2" t="inlineStr"/>
+      <c r="AE141" s="2" t="inlineStr"/>
+      <c r="AF141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG141" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH141" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>J-00141</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>ONLINE BEWERBEN</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>ONLINE BEWERBEN</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr"/>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>DE
+Einfach bewerben
+Bewerbung aktuell möglich
+Initiativbewerbung Studenten (m/w/d)
+e.solutions GmbH
+Ingolstadt
+* Pflichtfeld
+Persönliche Angaben
+Ihre Kontaktdaten
+Anrede*
+erforderlich
+Anrede wählen...
+Herr
+Frau
+Divers
+Vorname*
+erforderlich
+Nachname*
+erforderlich
+Straße und Hausnummer*
+erforderlich
+Postleitzahl*
+erforderlich
+Wohnort*
+erforderlich
+E-Mail Adresse*
+erforderlich
+Telefonnummer*
+erforderlich
+Lebenslauf
+Stationen Ihres Berufswegs
+Lebenslauf*
+erforderlich
+Datei auswählen oder hierher z</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>https://esolutions.onlyfy.jobs/application/apply/9l94ga1zx7ect8wlibk2izu282i3ka</t>
+        </is>
+      </c>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N142" s="2" t="n"/>
+      <c r="O142" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q142" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R142" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S142" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V142" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W142" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/endobit software solutions_ONLINE BEWERBEN.html</t>
+        </is>
+      </c>
+      <c r="X142" s="2" t="inlineStr">
+        <is>
+          <t>werkstudent</t>
+        </is>
+      </c>
+      <c r="Y142" s="2" t="inlineStr">
+        <is>
+          <t>developer</t>
+        </is>
+      </c>
+      <c r="Z142" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA142" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB142" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="AC142" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD142" s="2" t="inlineStr"/>
+      <c r="AE142" s="2" t="inlineStr"/>
+      <c r="AF142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG142" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH142" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>J-00142</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent (m/w/d) – HMI</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent (m/w/d) – HMI</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>IT-Ausbildung &amp; Studium</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>java, angular, kotlin</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>SOFTWARE by e.solutions
+WIR bei e.solutions
+DU bei e.solutions
+KONTAKT
+Werkstudent (m/w/d) – HMI
+Studierende Erlangen xwp8lq2c
+JETZT ONLINE BEWERBEN
+Die Zukunft des Autos findet im Innenraum statt. Die Software dazu entwickeln wir! Als Joint Venture der CARIAD SE und der Elektrobit Automotive GmbH entwickeln wir hochkomplexe Lösungen für die Kommunikation im und aus dem Auto. Für unsere Kunden aus dem VW-Konzern gestalten wir Frameworks, Applikationen und graphische Benutzeroberflächen und fü</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs/details/werkstudent-mwd-hmi</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N143" s="2" t="n"/>
+      <c r="O143" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P143" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q143" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R143" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S143" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V143" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W143" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/endobit software solutions_Werkstudent _m_w_d_ _ HMI.html</t>
+        </is>
+      </c>
+      <c r="X143" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y143" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z143" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA143" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB143" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="AC143" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD143" s="2" t="inlineStr"/>
+      <c r="AE143" s="2" t="inlineStr"/>
+      <c r="AF143" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG143" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH143" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI143" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ143" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK143" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>J-00143</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>ONLINE BEWERBEN</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>ONLINE BEWERBEN</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr"/>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE
+Einfach bewerben
+Bewerbung aktuell möglich
+Werkstudent (m/w/d) – HMI
+e.solutions GmbH
+Erlangen
+Vor Ort &amp; Home-Office
+* Pflichtfeld
+Persönliche Angaben
+Ihre Kontaktdaten
+Anrede*
+erforderlich
+Anrede wählen...
+Herr
+Frau
+Divers
+Vorname*
+erforderlich
+Nachname*
+erforderlich
+Straße und Hausnummer*
+erforderlich
+Postleitzahl*
+erforderlich
+Wohnort*
+erforderlich
+E-Mail Adresse*
+erforderlich
+Telefonnummer*
+erforderlich
+Lebenslauf
+Stationen Ihres Berufswegs
+Lebenslauf*
+erforderlich
+Datei auswählen oder </t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>https://esolutions.onlyfy.jobs/application/apply/gh8tog83ium0bj9zql9rsdj8h3nycn</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N144" s="2" t="n"/>
+      <c r="O144" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q144" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R144" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S144" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V144" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W144" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/endobit software solutions_ONLINE BEWERBEN.html</t>
+        </is>
+      </c>
+      <c r="X144" s="2" t="inlineStr">
+        <is>
+          <t>werkstudent</t>
+        </is>
+      </c>
+      <c r="Y144" s="2" t="inlineStr">
+        <is>
+          <t>developer</t>
+        </is>
+      </c>
+      <c r="Z144" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA144" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB144" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="AC144" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD144" s="2" t="inlineStr"/>
+      <c r="AE144" s="2" t="inlineStr"/>
+      <c r="AF144" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG144" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH144" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI144" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ144" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK144" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>J-00144</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent Flash Support (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent Flash Support (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>IT-Ausbildung &amp; Studium</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr"/>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>SOFTWARE by e.solutions
+WIR bei e.solutions
+DU bei e.solutions
+KONTAKT
+Werkstudent Flash Support (m/w/d)
+Studierende Ingolstadt bcec0drt
+JETZT ONLINE BEWERBEN
+Die Zukunft des Autos findet im Innenraum statt. Die Software dazu entwickeln wir! Als Joint Venture der CARIAD SE und der Elektrobit Automotive GmbH entwickeln wir hochkomplexe Lösungen für die Kommunikation im und aus dem Auto. Für unsere Kunden aus dem VW-Konzern gestalten wir Frameworks, Applikationen und graphische Benutzeroberfläc</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs/details/werkstudent-flash-support-mwd</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N145" s="2" t="n"/>
+      <c r="O145" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P145" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q145" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R145" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S145" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V145" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W145" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/endobit software solutions_Werkstudent Flash Support _m_w_d.html</t>
+        </is>
+      </c>
+      <c r="X145" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y145" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z145" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA145" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB145" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent</t>
+        </is>
+      </c>
+      <c r="AC145" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD145" s="2" t="inlineStr"/>
+      <c r="AE145" s="2" t="inlineStr"/>
+      <c r="AF145" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG145" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH145" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI145" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ145" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK145" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>J-00145</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>SecMail-Portal</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>SecMail-Portal</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr"/>
+      <c r="I146" s="2" t="inlineStr"/>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>https://secmail.esolutions.de/</t>
+        </is>
+      </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N146" s="2" t="n"/>
+      <c r="O146" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q146" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R146" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S146" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V146" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W146" s="2" t="inlineStr"/>
+      <c r="X146" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y146" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z146" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA146" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB146" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC146" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD146" s="2" t="inlineStr"/>
+      <c r="AE146" s="2" t="inlineStr"/>
+      <c r="AF146" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG146" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH146" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI146" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ146" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK146" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>J-00146</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>eso.IT.Support</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>eso.IT.Support</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr"/>
+      <c r="I147" s="2" t="inlineStr"/>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>mailto:eso.it.support@esolutions.de</t>
+        </is>
+      </c>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N147" s="2" t="n"/>
+      <c r="O147" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P147" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q147" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R147" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S147" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V147" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W147" s="2" t="inlineStr"/>
+      <c r="X147" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y147" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="Z147" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA147" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB147" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC147" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD147" s="2" t="inlineStr"/>
+      <c r="AE147" s="2" t="inlineStr"/>
+      <c r="AF147" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG147" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH147" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI147" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ147" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK147" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>J-00147</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>SOFTWARE by e.solutions</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>SOFTWARE by e.solutions</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr"/>
+      <c r="I148" s="2" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/software-by-esolutions</t>
+        </is>
+      </c>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="n"/>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q148" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R148" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S148" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V148" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W148" s="2" t="inlineStr"/>
+      <c r="X148" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y148" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z148" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA148" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB148" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC148" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD148" s="2" t="inlineStr"/>
+      <c r="AE148" s="2" t="inlineStr"/>
+      <c r="AF148" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG148" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH148" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI148" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ148" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK148" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>J-00148</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Infotainmentsystem</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Infotainmentsystem</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr"/>
+      <c r="I149" s="2" t="inlineStr"/>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/software-by-esolutions/infotainmentsystem</t>
+        </is>
+      </c>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>endobit software solutions</t>
+        </is>
+      </c>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>endobitsoftwaresolutions</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N149" s="2" t="n"/>
+      <c r="O149" s="2" t="inlineStr">
+        <is>
+          <t>Wittelsbacherstraße 1</t>
+        </is>
+      </c>
+      <c r="P149" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 98814800</t>
+        </is>
+      </c>
+      <c r="Q149" s="2" t="inlineStr">
+        <is>
+          <t>info@esolutions.de</t>
+        </is>
+      </c>
+      <c r="R149" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S149" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T149" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/du-bei-esolutions/jobs</t>
+        </is>
+      </c>
+      <c r="U149" s="2" t="inlineStr">
+        <is>
+          <t>https://www.esolutions.de/de/</t>
+        </is>
+      </c>
+      <c r="V149" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/endobit software solutions_career.html</t>
+        </is>
+      </c>
+      <c r="W149" s="2" t="inlineStr"/>
+      <c r="X149" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y149" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="Z149" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA149" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB149" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC149" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD149" s="2" t="inlineStr"/>
+      <c r="AE149" s="2" t="inlineStr"/>
+      <c r="AF149" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AG149" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH149" s="2" t="n">
+        <v>2379</v>
+      </c>
+      <c r="AI149" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ149" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+      <c r="AK149" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21753,7 +23682,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>137</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2">
@@ -21764,7 +23693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-14 15:34</t>
+          <t>2026-05-14 15:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Junior IT Jobs - 159 jobs (15:35)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
+++ b/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK149"/>
+  <dimension ref="A1:AK160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23661,6 +23661,1805 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>J-00149</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Alle Stellenangebote</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Alle Stellenangebote</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>IT-Ausbildung &amp; Studium</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr"/>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>Handwerk
+​
+Technischer Projektmitarbeiter im SHK-Bereich (m/w/d)
+​
+Ausbildungsplatz für 2026: Kaufmann bzw. Kauffrau für Büromanagement
+Sonstige Berufe
+​
+Reinigungskraft (m/w/d) für die Hauptverwaltung der HWK in Bayreuth</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.hwk-oberfranken.de/_/joblist</t>
+        </is>
+      </c>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>Arbeitsbeschaffungsstelle des Handwerks eG</t>
+        </is>
+      </c>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>arbeitsbeschaffungsstelledeshandwerks</t>
+        </is>
+      </c>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="N150" s="2" t="n"/>
+      <c r="O150" s="2" t="inlineStr">
+        <is>
+          <t>Zollnerstraße 217</t>
+        </is>
+      </c>
+      <c r="P150" s="2" t="inlineStr">
+        <is>
+          <t>+49 951 200452</t>
+        </is>
+      </c>
+      <c r="Q150" s="2" t="inlineStr">
+        <is>
+          <t>info@hwk-oberfranken.de</t>
+        </is>
+      </c>
+      <c r="R150" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S150" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T150" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.hwk-oberfranken.de</t>
+        </is>
+      </c>
+      <c r="U150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hwk-oberfranken.de/artikel/das-neue-bildungszentrum-bamberg-72,0,3151.html</t>
+        </is>
+      </c>
+      <c r="V150" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Arbeitsbeschaffungsstelle des Handwerks eG_career.html</t>
+        </is>
+      </c>
+      <c r="W150" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Arbeitsbeschaffungsstelle des Handwerks _Alle Stellenangebote.html</t>
+        </is>
+      </c>
+      <c r="X150" s="2" t="inlineStr">
+        <is>
+          <t>ausbildung</t>
+        </is>
+      </c>
+      <c r="Y150" s="2" t="inlineStr">
+        <is>
+          <t>projekt</t>
+        </is>
+      </c>
+      <c r="Z150" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA150" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB150" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung</t>
+        </is>
+      </c>
+      <c r="AC150" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD150" s="2" t="inlineStr"/>
+      <c r="AE150" s="2" t="inlineStr"/>
+      <c r="AF150" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:27</t>
+        </is>
+      </c>
+      <c r="AG150" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH150" s="2" t="n">
+        <v>2413</v>
+      </c>
+      <c r="AI150" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ150" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:27</t>
+        </is>
+      </c>
+      <c r="AK150" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>J-00150</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>zur Website</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>zur Website</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>Vor Ort</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr"/>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>Startseite der Handwerkskammer für Oberfranken
+Karussell-Element
+Karussell-Element anhalten
+Anzeigen von Karussell-Element 1
+Anzeigen von Karussell-Element 2
+Podiumsdiskussion
+Frauen im Handwerk: Vernetzung und Sichtbarkeit als Weg
+HWK-Podiumsdiskussion zum Projekt „Mutige Frauen – starkes Handwerk“ – Erkenntnisse aus Umfrage und konkrete Handlungsempfehlungen
+HWK für Oberfranken / Stefan Dörfler
+Frauen im Handwerk: Vernetzung und Sichtbarkeit als Weg
+Vorheriges Karussell-Element
+Nachfolgendes</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hwk-oberfranken.de/</t>
+        </is>
+      </c>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>Arbeitsbeschaffungsstelle des Handwerks eG</t>
+        </is>
+      </c>
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>arbeitsbeschaffungsstelledeshandwerks</t>
+        </is>
+      </c>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="N151" s="2" t="n"/>
+      <c r="O151" s="2" t="inlineStr">
+        <is>
+          <t>Zollnerstraße 217</t>
+        </is>
+      </c>
+      <c r="P151" s="2" t="inlineStr">
+        <is>
+          <t>+49 951 200452</t>
+        </is>
+      </c>
+      <c r="Q151" s="2" t="inlineStr">
+        <is>
+          <t>info@hwk-oberfranken.de</t>
+        </is>
+      </c>
+      <c r="R151" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S151" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T151" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.hwk-oberfranken.de</t>
+        </is>
+      </c>
+      <c r="U151" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hwk-oberfranken.de/artikel/das-neue-bildungszentrum-bamberg-72,0,3151.html</t>
+        </is>
+      </c>
+      <c r="V151" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Arbeitsbeschaffungsstelle des Handwerks eG_career.html</t>
+        </is>
+      </c>
+      <c r="W151" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Arbeitsbeschaffungsstelle des Handwerks _zur Website.html</t>
+        </is>
+      </c>
+      <c r="X151" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y151" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z151" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA151" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB151" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="AC151" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD151" s="2" t="inlineStr"/>
+      <c r="AE151" s="2" t="inlineStr"/>
+      <c r="AF151" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:27</t>
+        </is>
+      </c>
+      <c r="AG151" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH151" s="2" t="n">
+        <v>2413</v>
+      </c>
+      <c r="AI151" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ151" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:27</t>
+        </is>
+      </c>
+      <c r="AK151" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>J-00151</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Saved jobs
+(0)</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Saved jobs
+(0)</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr"/>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>-
+Saved Jobs
+your saved jobs
+skip this widget
+Join our talent community
+Interested in staying connected? Sign up for our talent community to receive updates on life at Cencora and to learn about the impact our team members are making on delivering the future of healthcare.
+Sign up</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.cencora.com/us/en/jobcart</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>Alliance Healthcare Deutschland GmbH - Niederlassung Nürnberg</t>
+        </is>
+      </c>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>alliancehealthcaredeutschlandniederlassungnürnberg</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N152" s="2" t="n"/>
+      <c r="O152" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg
+2</t>
+        </is>
+      </c>
+      <c r="P152" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 52740</t>
+        </is>
+      </c>
+      <c r="Q152" s="2" t="n"/>
+      <c r="R152" s="2" t="n"/>
+      <c r="S152" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T152" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cencora.com/careers</t>
+        </is>
+      </c>
+      <c r="U152" s="2" t="inlineStr">
+        <is>
+          <t>https://www.alliance-healthcare.com</t>
+        </is>
+      </c>
+      <c r="V152" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Alliance Healthcare Deutschland GmbH - Niederlassung Nürnberg_career.html</t>
+        </is>
+      </c>
+      <c r="W152" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Alliance Healthcare Deutschland GmbH - N_Saved jobs
+_0.html</t>
+        </is>
+      </c>
+      <c r="X152" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y152" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z152" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA152" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB152" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC152" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD152" s="2" t="inlineStr"/>
+      <c r="AE152" s="2" t="inlineStr"/>
+      <c r="AF152" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:38</t>
+        </is>
+      </c>
+      <c r="AG152" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH152" s="2" t="n">
+        <v>2402</v>
+      </c>
+      <c r="AI152" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ152" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:38</t>
+        </is>
+      </c>
+      <c r="AK152" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>J-00152</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Manager, Local Pharmacovigilance</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Manager, Local Pharmacovigilance</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>UX/UI Design</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr"/>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>-
+Search job title
+Location
+Search
+Careers at the
+center of health
+Manager, Local Pharmacovigilance
+Location:
+Mechelen, Belgium
+Category:
+Consulting
+widget:
+Full time
+Posted Date:
+July 23rd 2025
+Job ID:
+R2513984
+Apply now
+Save
+About Cencora
+Our team members are at the heart of everything we do. At Cencora, we are united in our responsibility to create healthier futures, and every person here is essential to us being able to deliver on that purpose. If you want to make a difference at the center</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.cencora.com/us/en/job/R2513984/Manager-Local-Pharmacovigilance</t>
+        </is>
+      </c>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>Alliance Healthcare Deutschland GmbH - Niederlassung Nürnberg</t>
+        </is>
+      </c>
+      <c r="L153" s="2" t="inlineStr">
+        <is>
+          <t>alliancehealthcaredeutschlandniederlassungnürnberg</t>
+        </is>
+      </c>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N153" s="2" t="n"/>
+      <c r="O153" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg
+2</t>
+        </is>
+      </c>
+      <c r="P153" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 52740</t>
+        </is>
+      </c>
+      <c r="Q153" s="2" t="n"/>
+      <c r="R153" s="2" t="n"/>
+      <c r="S153" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T153" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cencora.com/careers</t>
+        </is>
+      </c>
+      <c r="U153" s="2" t="inlineStr">
+        <is>
+          <t>https://www.alliance-healthcare.com</t>
+        </is>
+      </c>
+      <c r="V153" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Alliance Healthcare Deutschland GmbH - Niederlassung Nürnberg_career.html</t>
+        </is>
+      </c>
+      <c r="W153" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Alliance Healthcare Deutschland GmbH - N_Manager_ Local Pharmacovigilance.html</t>
+        </is>
+      </c>
+      <c r="X153" s="2" t="inlineStr">
+        <is>
+          <t>junior</t>
+        </is>
+      </c>
+      <c r="Y153" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="Z153" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA153" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>J-00153</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Zu den Jobs</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Zu den Jobs</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr"/>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Create an alertAnd get notified by email as soon as a job matches with your criteria.NameLabel*CadenceDailyWeeklyYour criteria Create Cancel</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>https://dkv-mobility.csod.com/ux/ats/careersite/10/home?c=dkv-mobility</t>
+        </is>
+      </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>DKV Deutsche Krankenversicherung Peter Meyer</t>
+        </is>
+      </c>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>dkvdeutschekrankenversicherungpetermeyer</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="n"/>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>Nägelsbachstraße 25</t>
+        </is>
+      </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 206411</t>
+        </is>
+      </c>
+      <c r="Q154" s="2" t="n"/>
+      <c r="R154" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S154" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="U154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/company/dkv-mobility-group/peter-meier</t>
+        </is>
+      </c>
+      <c r="V154" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/DKV Deutsche Krankenversicherung Peter Meyer_career.html</t>
+        </is>
+      </c>
+      <c r="W154" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/DKV Deutsche Krankenversicherung Peter M_Zu den Jobs.html</t>
+        </is>
+      </c>
+      <c r="X154" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y154" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z154" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA154" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB154" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC154" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD154" s="2" t="inlineStr"/>
+      <c r="AE154" s="2" t="inlineStr"/>
+      <c r="AF154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AG154" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH154" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="AI154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AK154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>J-00154</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Jetzt Tech gestalten</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Jetzt Tech gestalten</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>node.js, kafka, kanban, sap, dynamics, java, agile, bash, python, swift, jira, javascript, go, scrum, kotlin, scala</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hero-level_2
+            Hero
+            TECH HEROES
+            text-size-headline-h2
+            We need your superpower!
+ </t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/de/career/our-stories/tech-heroes</t>
+        </is>
+      </c>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>DKV Deutsche Krankenversicherung Peter Meyer</t>
+        </is>
+      </c>
+      <c r="L155" s="2" t="inlineStr">
+        <is>
+          <t>dkvdeutschekrankenversicherungpetermeyer</t>
+        </is>
+      </c>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N155" s="2" t="n"/>
+      <c r="O155" s="2" t="inlineStr">
+        <is>
+          <t>Nägelsbachstraße 25</t>
+        </is>
+      </c>
+      <c r="P155" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 206411</t>
+        </is>
+      </c>
+      <c r="Q155" s="2" t="n"/>
+      <c r="R155" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S155" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T155" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="U155" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/company/dkv-mobility-group/peter-meier</t>
+        </is>
+      </c>
+      <c r="V155" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/DKV Deutsche Krankenversicherung Peter Meyer_career.html</t>
+        </is>
+      </c>
+      <c r="W155" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/DKV Deutsche Krankenversicherung Peter M_Jetzt Tech gestalten.html</t>
+        </is>
+      </c>
+      <c r="X155" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y155" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z155" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA155" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB155" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="AC155" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD155" s="2" t="inlineStr"/>
+      <c r="AE155" s="2" t="inlineStr"/>
+      <c r="AF155" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AG155" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH155" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="AI155" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ155" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AK155" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>J-00155</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Jetzt durchstarten</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Jetzt durchstarten</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Systemadministration</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>Teilzeit</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr"/>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hero-level_2
+            Hero
+            Erste Berufserfahrung sammelnbei DKV Mobility
+            text-size-headline-h2
+    </t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/de/career/working-at-dkv-mobility/youth-learning</t>
+        </is>
+      </c>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>DKV Deutsche Krankenversicherung Peter Meyer</t>
+        </is>
+      </c>
+      <c r="L156" s="2" t="inlineStr">
+        <is>
+          <t>dkvdeutschekrankenversicherungpetermeyer</t>
+        </is>
+      </c>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="n"/>
+      <c r="O156" s="2" t="inlineStr">
+        <is>
+          <t>Nägelsbachstraße 25</t>
+        </is>
+      </c>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 206411</t>
+        </is>
+      </c>
+      <c r="Q156" s="2" t="n"/>
+      <c r="R156" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S156" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="U156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/company/dkv-mobility-group/peter-meier</t>
+        </is>
+      </c>
+      <c r="V156" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/DKV Deutsche Krankenversicherung Peter Meyer_career.html</t>
+        </is>
+      </c>
+      <c r="W156" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/DKV Deutsche Krankenversicherung Peter M_Jetzt durchstarten.html</t>
+        </is>
+      </c>
+      <c r="X156" s="2" t="inlineStr">
+        <is>
+          <t>praktikant</t>
+        </is>
+      </c>
+      <c r="Y156" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z156" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA156" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB156" s="2" t="inlineStr">
+        <is>
+          <t>Teilzeit</t>
+        </is>
+      </c>
+      <c r="AC156" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD156" s="2" t="inlineStr"/>
+      <c r="AE156" s="2" t="inlineStr"/>
+      <c r="AF156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AG156" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH156" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="AI156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AK156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>J-00156</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Social Stories lesen</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Social Stories lesen</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>UX/UI Design</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr"/>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hero-level_2
+            Hero
+            Geschichten aus unseremAlltag – Das macht uns aus
+            text-size-headline-h2
+</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/de/career/our-stories/social-stories</t>
+        </is>
+      </c>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>DKV Deutsche Krankenversicherung Peter Meyer</t>
+        </is>
+      </c>
+      <c r="L157" s="2" t="inlineStr">
+        <is>
+          <t>dkvdeutschekrankenversicherungpetermeyer</t>
+        </is>
+      </c>
+      <c r="M157" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N157" s="2" t="n"/>
+      <c r="O157" s="2" t="inlineStr">
+        <is>
+          <t>Nägelsbachstraße 25</t>
+        </is>
+      </c>
+      <c r="P157" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 206411</t>
+        </is>
+      </c>
+      <c r="Q157" s="2" t="n"/>
+      <c r="R157" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S157" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="U157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/company/dkv-mobility-group/peter-meier</t>
+        </is>
+      </c>
+      <c r="V157" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/DKV Deutsche Krankenversicherung Peter Meyer_career.html</t>
+        </is>
+      </c>
+      <c r="W157" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/DKV Deutsche Krankenversicherung Peter M_Social Stories lesen.html</t>
+        </is>
+      </c>
+      <c r="X157" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y157" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z157" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA157" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB157" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="AC157" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD157" s="2" t="inlineStr"/>
+      <c r="AE157" s="2" t="inlineStr"/>
+      <c r="AF157" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AG157" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH157" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="AI157" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ157" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AK157" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>J-00157</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>eMobility Support00800 24 007 365</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>eMobility Support00800 24 007 365</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr"/>
+      <c r="I158" s="2" t="inlineStr"/>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>tel:08003583583</t>
+        </is>
+      </c>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>DKV Deutsche Krankenversicherung Peter Meyer</t>
+        </is>
+      </c>
+      <c r="L158" s="2" t="inlineStr">
+        <is>
+          <t>dkvdeutschekrankenversicherungpetermeyer</t>
+        </is>
+      </c>
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N158" s="2" t="n"/>
+      <c r="O158" s="2" t="inlineStr">
+        <is>
+          <t>Nägelsbachstraße 25</t>
+        </is>
+      </c>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 206411</t>
+        </is>
+      </c>
+      <c r="Q158" s="2" t="n"/>
+      <c r="R158" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S158" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="U158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/company/dkv-mobility-group/peter-meier</t>
+        </is>
+      </c>
+      <c r="V158" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/DKV Deutsche Krankenversicherung Peter Meyer_career.html</t>
+        </is>
+      </c>
+      <c r="W158" s="2" t="inlineStr"/>
+      <c r="X158" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y158" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="Z158" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA158" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB158" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC158" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD158" s="2" t="inlineStr"/>
+      <c r="AE158" s="2" t="inlineStr"/>
+      <c r="AF158" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AG158" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH158" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="AI158" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ158" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AK158" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>J-00158</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Hinweisgebersystem</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Hinweisgebersystem</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr"/>
+      <c r="I159" s="2" t="inlineStr"/>
+      <c r="J159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/whistleblowing-system</t>
+        </is>
+      </c>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>DKV Deutsche Krankenversicherung Peter Meyer</t>
+        </is>
+      </c>
+      <c r="L159" s="2" t="inlineStr">
+        <is>
+          <t>dkvdeutschekrankenversicherungpetermeyer</t>
+        </is>
+      </c>
+      <c r="M159" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N159" s="2" t="n"/>
+      <c r="O159" s="2" t="inlineStr">
+        <is>
+          <t>Nägelsbachstraße 25</t>
+        </is>
+      </c>
+      <c r="P159" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 206411</t>
+        </is>
+      </c>
+      <c r="Q159" s="2" t="n"/>
+      <c r="R159" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S159" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="U159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/company/dkv-mobility-group/peter-meier</t>
+        </is>
+      </c>
+      <c r="V159" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/DKV Deutsche Krankenversicherung Peter Meyer_career.html</t>
+        </is>
+      </c>
+      <c r="W159" s="2" t="inlineStr"/>
+      <c r="X159" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y159" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="Z159" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA159" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB159" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC159" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD159" s="2" t="inlineStr"/>
+      <c r="AE159" s="2" t="inlineStr"/>
+      <c r="AF159" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AG159" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH159" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="AI159" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ159" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AK159" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>J-00159</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Cookie Settings</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Cookie Settings</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr"/>
+      <c r="I160" s="2" t="inlineStr"/>
+      <c r="J160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>DKV Deutsche Krankenversicherung Peter Meyer</t>
+        </is>
+      </c>
+      <c r="L160" s="2" t="inlineStr">
+        <is>
+          <t>dkvdeutschekrankenversicherungpetermeyer</t>
+        </is>
+      </c>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N160" s="2" t="n"/>
+      <c r="O160" s="2" t="inlineStr">
+        <is>
+          <t>Nägelsbachstraße 25</t>
+        </is>
+      </c>
+      <c r="P160" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 206411</t>
+        </is>
+      </c>
+      <c r="Q160" s="2" t="n"/>
+      <c r="R160" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S160" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/de/karriere</t>
+        </is>
+      </c>
+      <c r="U160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dkv-mobility.com/uk/en/company/dkv-mobility-group/peter-meier</t>
+        </is>
+      </c>
+      <c r="V160" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/DKV Deutsche Krankenversicherung Peter Meyer_career.html</t>
+        </is>
+      </c>
+      <c r="W160" s="2" t="inlineStr"/>
+      <c r="X160" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y160" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z160" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA160" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB160" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC160" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD160" s="2" t="inlineStr"/>
+      <c r="AE160" s="2" t="inlineStr"/>
+      <c r="AF160" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AG160" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH160" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="AI160" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ160" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+      <c r="AK160" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:35:59</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23682,7 +25481,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>148</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Junior IT Jobs - 186 jobs (15:36)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
+++ b/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK160"/>
+  <dimension ref="A1:AK187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -25460,6 +25460,4199 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>J-00160</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Pharmazie
+Ob angestellt in der öffentliche Apotheke, Krankenhausapotheke, Industrie oder der Schritt in die Selbstständigkeit . Finde heraus, wie du deinen Platz in der faszinierenden Welt der Pharmaz</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Pharmazie
+Ob angestellt in der öffentliche Apotheke, Krankenhausapotheke, Industrie oder der Schritt in die Selbstständigkeit . Finde heraus, wie du deinen Platz in der faszinierenden Welt der Pharmaz</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr"/>
+      <c r="I161" s="2" t="inlineStr"/>
+      <c r="J161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler/apotheker-gehalt-und-work-life-balance</t>
+        </is>
+      </c>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L161" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N161" s="2" t="n"/>
+      <c r="O161" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P161" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q161" s="2" t="n"/>
+      <c r="R161" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S161" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V161" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W161" s="2" t="inlineStr"/>
+      <c r="X161" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y161" s="2" t="inlineStr">
+        <is>
+          <t>sap</t>
+        </is>
+      </c>
+      <c r="Z161" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA161" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB161" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC161" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD161" s="2" t="inlineStr"/>
+      <c r="AE161" s="2" t="inlineStr"/>
+      <c r="AF161" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG161" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH161" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI161" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ161" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK161" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>J-00161</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Veterinärmedizin
+Welche Arbeitsmodelle unterstützen eine ausgewogene Work-Life-Balance?
+Ob Kleintier-, oder Großtierpraxis, ob Forschung, Industrie oder öffentlicher Dienst – hier bekommst du Orientie</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Veterinärmedizin
+Welche Arbeitsmodelle unterstützen eine ausgewogene Work-Life-Balance?
+Ob Kleintier-, oder Großtierpraxis, ob Forschung, Industrie oder öffentlicher Dienst – hier bekommst du Orientie</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr"/>
+      <c r="I162" s="2" t="inlineStr"/>
+      <c r="J162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler/tierarzt-gehalt-und-work-life-balance</t>
+        </is>
+      </c>
+      <c r="K162" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L162" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N162" s="2" t="n"/>
+      <c r="O162" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P162" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q162" s="2" t="n"/>
+      <c r="R162" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S162" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V162" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W162" s="2" t="inlineStr"/>
+      <c r="X162" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y162" s="2" t="inlineStr">
+        <is>
+          <t>erp</t>
+        </is>
+      </c>
+      <c r="Z162" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA162" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB162" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC162" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD162" s="2" t="inlineStr"/>
+      <c r="AE162" s="2" t="inlineStr"/>
+      <c r="AF162" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG162" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH162" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI162" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ162" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK162" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>J-00162</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Psychologische Psychotherapie
+Die psychologische Psychotherapie bietet vielfältige Karrierewege. Hier erhältst du einen Überblick was dich fachlich, organisatorisch und persönlich in diesem Berufsfeld</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Psychologische Psychotherapie
+Die psychologische Psychotherapie bietet vielfältige Karrierewege. Hier erhältst du einen Überblick was dich fachlich, organisatorisch und persönlich in diesem Berufsfeld</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr"/>
+      <c r="I163" s="2" t="inlineStr"/>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler/psychologischer-psychotherapeut-gehalt-und-work-life-balance</t>
+        </is>
+      </c>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L163" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N163" s="2" t="n"/>
+      <c r="O163" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P163" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q163" s="2" t="n"/>
+      <c r="R163" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S163" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V163" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W163" s="2" t="inlineStr"/>
+      <c r="X163" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y163" s="2" t="inlineStr">
+        <is>
+          <t>api</t>
+        </is>
+      </c>
+      <c r="Z163" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA163" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB163" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC163" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD163" s="2" t="inlineStr"/>
+      <c r="AE163" s="2" t="inlineStr"/>
+      <c r="AF163" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG163" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH163" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI163" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ163" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK163" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>J-00163</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Online Banking</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Online Banking</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr"/>
+      <c r="I164" s="2" t="inlineStr"/>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t>https://banking.apobank.de/auth/login</t>
+        </is>
+      </c>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L164" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N164" s="2" t="n"/>
+      <c r="O164" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P164" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q164" s="2" t="n"/>
+      <c r="R164" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S164" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V164" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W164" s="2" t="inlineStr"/>
+      <c r="X164" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y164" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z164" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA164" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB164" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC164" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD164" s="2" t="inlineStr"/>
+      <c r="AE164" s="2" t="inlineStr"/>
+      <c r="AF164" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG164" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH164" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI164" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ164" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK164" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>J-00164</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr"/>
+      <c r="I165" s="2" t="inlineStr"/>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/unsere-leistungen/konto-karte/online-banking</t>
+        </is>
+      </c>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L165" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N165" s="2" t="n"/>
+      <c r="O165" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P165" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q165" s="2" t="n"/>
+      <c r="R165" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S165" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V165" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W165" s="2" t="inlineStr"/>
+      <c r="X165" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y165" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z165" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA165" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB165" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC165" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD165" s="2" t="inlineStr"/>
+      <c r="AE165" s="2" t="inlineStr"/>
+      <c r="AF165" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG165" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH165" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI165" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ165" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK165" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>J-00165</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking Hilfe</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking Hilfe</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr"/>
+      <c r="I166" s="2" t="inlineStr"/>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/online-und-mobile-banking</t>
+        </is>
+      </c>
+      <c r="K166" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L166" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M166" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N166" s="2" t="n"/>
+      <c r="O166" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P166" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q166" s="2" t="n"/>
+      <c r="R166" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S166" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V166" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W166" s="2" t="inlineStr"/>
+      <c r="X166" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y166" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z166" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA166" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB166" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC166" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD166" s="2" t="inlineStr"/>
+      <c r="AE166" s="2" t="inlineStr"/>
+      <c r="AF166" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG166" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH166" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI166" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ166" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK166" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>J-00166</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Telefon-Banking</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Telefon-Banking</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr"/>
+      <c r="I167" s="2" t="inlineStr"/>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/unsere-leistungen/konto-karte/telefon-banking</t>
+        </is>
+      </c>
+      <c r="K167" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L167" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M167" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N167" s="2" t="n"/>
+      <c r="O167" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P167" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q167" s="2" t="n"/>
+      <c r="R167" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S167" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V167" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W167" s="2" t="inlineStr"/>
+      <c r="X167" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y167" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z167" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA167" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB167" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC167" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD167" s="2" t="inlineStr"/>
+      <c r="AE167" s="2" t="inlineStr"/>
+      <c r="AF167" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG167" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH167" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI167" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ167" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK167" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>J-00167</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Mobile-Banking</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Mobile-Banking</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr"/>
+      <c r="I168" s="2" t="inlineStr"/>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/unsere-leistungen/konto-karte/mobile-banking</t>
+        </is>
+      </c>
+      <c r="K168" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L168" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N168" s="2" t="n"/>
+      <c r="O168" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P168" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q168" s="2" t="n"/>
+      <c r="R168" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S168" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V168" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W168" s="2" t="inlineStr"/>
+      <c r="X168" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y168" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z168" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA168" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB168" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC168" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD168" s="2" t="inlineStr"/>
+      <c r="AE168" s="2" t="inlineStr"/>
+      <c r="AF168" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG168" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH168" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI168" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ168" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK168" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>J-00168</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Banking-Software</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Banking-Software</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr"/>
+      <c r="I169" s="2" t="inlineStr"/>
+      <c r="J169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/unsere-leistungen/konto-karte/banking-software</t>
+        </is>
+      </c>
+      <c r="K169" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L169" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N169" s="2" t="n"/>
+      <c r="O169" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P169" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q169" s="2" t="n"/>
+      <c r="R169" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S169" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V169" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W169" s="2" t="inlineStr"/>
+      <c r="X169" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y169" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z169" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA169" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB169" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC169" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD169" s="2" t="inlineStr"/>
+      <c r="AE169" s="2" t="inlineStr"/>
+      <c r="AF169" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG169" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH169" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI169" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ169" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK169" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>J-00169</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Telefon-Banking</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Telefon-Banking</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr"/>
+      <c r="I170" s="2" t="inlineStr"/>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/unsere-leistungen/weiterleitungsseite-telefon-banking</t>
+        </is>
+      </c>
+      <c r="K170" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L170" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M170" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N170" s="2" t="n"/>
+      <c r="O170" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P170" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q170" s="2" t="n"/>
+      <c r="R170" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S170" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V170" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W170" s="2" t="inlineStr"/>
+      <c r="X170" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y170" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z170" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA170" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB170" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC170" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD170" s="2" t="inlineStr"/>
+      <c r="AE170" s="2" t="inlineStr"/>
+      <c r="AF170" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG170" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH170" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI170" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ170" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK170" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>J-00170</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr"/>
+      <c r="I171" s="2" t="inlineStr"/>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/unsere-leistungen/weiterleitungsseite-online-banking</t>
+        </is>
+      </c>
+      <c r="K171" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L171" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N171" s="2" t="n"/>
+      <c r="O171" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P171" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q171" s="2" t="n"/>
+      <c r="R171" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S171" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V171" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W171" s="2" t="inlineStr"/>
+      <c r="X171" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y171" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z171" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA171" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB171" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC171" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD171" s="2" t="inlineStr"/>
+      <c r="AE171" s="2" t="inlineStr"/>
+      <c r="AF171" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG171" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH171" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI171" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ171" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK171" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>J-00171</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking - Login und Informationen</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Online-Banking - Login und Informationen</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr"/>
+      <c r="I172" s="2" t="inlineStr"/>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/onlinebanking</t>
+        </is>
+      </c>
+      <c r="K172" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L172" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N172" s="2" t="n"/>
+      <c r="O172" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P172" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q172" s="2" t="n"/>
+      <c r="R172" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S172" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V172" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W172" s="2" t="inlineStr"/>
+      <c r="X172" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y172" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z172" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA172" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB172" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC172" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD172" s="2" t="inlineStr"/>
+      <c r="AE172" s="2" t="inlineStr"/>
+      <c r="AF172" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG172" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH172" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI172" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ172" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK172" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>J-00172</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>Digitalisierung in der Praxis</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Digitalisierung in der Praxis</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr"/>
+      <c r="I173" s="2" t="inlineStr"/>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/praxis-apotheke/optimieren/die-digitale-praxis</t>
+        </is>
+      </c>
+      <c r="K173" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L173" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M173" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N173" s="2" t="n"/>
+      <c r="O173" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P173" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q173" s="2" t="n"/>
+      <c r="R173" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S173" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T173" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U173" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V173" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W173" s="2" t="inlineStr"/>
+      <c r="X173" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y173" s="2" t="inlineStr">
+        <is>
+          <t>digitalisierung</t>
+        </is>
+      </c>
+      <c r="Z173" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA173" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB173" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC173" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD173" s="2" t="inlineStr"/>
+      <c r="AE173" s="2" t="inlineStr"/>
+      <c r="AF173" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG173" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH173" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI173" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ173" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK173" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>J-00173</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Netzwerkpartner</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Netzwerkpartner</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr"/>
+      <c r="I174" s="2" t="inlineStr"/>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/praxis-apotheke/netzwerkpartner</t>
+        </is>
+      </c>
+      <c r="K174" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L174" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M174" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N174" s="2" t="n"/>
+      <c r="O174" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P174" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q174" s="2" t="n"/>
+      <c r="R174" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S174" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T174" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U174" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V174" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W174" s="2" t="inlineStr"/>
+      <c r="X174" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y174" s="2" t="inlineStr">
+        <is>
+          <t>netzwerk</t>
+        </is>
+      </c>
+      <c r="Z174" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA174" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB174" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC174" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD174" s="2" t="inlineStr"/>
+      <c r="AE174" s="2" t="inlineStr"/>
+      <c r="AF174" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG174" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH174" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI174" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ174" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK174" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>J-00174</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Selbständigkeit in vier Kapiteln</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Selbständigkeit in vier Kapiteln</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr"/>
+      <c r="I175" s="2" t="inlineStr"/>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/existenzgruendung/gruenderwissen/bausteine-selbstaendigkeit</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L175" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N175" s="2" t="n"/>
+      <c r="O175" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P175" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q175" s="2" t="n"/>
+      <c r="R175" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S175" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T175" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U175" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V175" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W175" s="2" t="inlineStr"/>
+      <c r="X175" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y175" s="2" t="inlineStr">
+        <is>
+          <t>api</t>
+        </is>
+      </c>
+      <c r="Z175" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA175" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB175" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC175" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD175" s="2" t="inlineStr"/>
+      <c r="AE175" s="2" t="inlineStr"/>
+      <c r="AF175" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG175" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH175" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI175" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ175" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK175" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>J-00175</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Aktuell: Förderprogramme für Versorgungseinrichtungen</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Aktuell: Förderprogramme für Versorgungseinrichtungen</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr"/>
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/firmenkunden/foerderung-fuer-krankenhaeuser</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L176" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M176" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N176" s="2" t="n"/>
+      <c r="O176" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P176" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q176" s="2" t="n"/>
+      <c r="R176" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S176" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V176" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W176" s="2" t="inlineStr"/>
+      <c r="X176" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y176" s="2" t="inlineStr">
+        <is>
+          <t>erp</t>
+        </is>
+      </c>
+      <c r="Z176" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA176" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB176" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC176" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD176" s="2" t="inlineStr"/>
+      <c r="AE176" s="2" t="inlineStr"/>
+      <c r="AF176" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG176" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH176" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI176" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ176" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK176" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>J-00176</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>Marktanalysten Versorgungsstrukturen</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Marktanalysten Versorgungsstrukturen</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr"/>
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/medizinische-versorgungsstrukturen/marktanalysten</t>
+        </is>
+      </c>
+      <c r="K177" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L177" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M177" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N177" s="2" t="n"/>
+      <c r="O177" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P177" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q177" s="2" t="n"/>
+      <c r="R177" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S177" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T177" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U177" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V177" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W177" s="2" t="inlineStr"/>
+      <c r="X177" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y177" s="2" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="Z177" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA177" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB177" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC177" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD177" s="2" t="inlineStr"/>
+      <c r="AE177" s="2" t="inlineStr"/>
+      <c r="AF177" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG177" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH177" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI177" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ177" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK177" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>J-00177</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Deutsches Netzwerk Versorgungsstrukturen</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Deutsches Netzwerk Versorgungsstrukturen</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr"/>
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/medizinische-versorgungsstrukturen/deutsches-netzwerk-versorgungsstrukturen</t>
+        </is>
+      </c>
+      <c r="K178" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L178" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M178" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N178" s="2" t="n"/>
+      <c r="O178" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P178" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q178" s="2" t="n"/>
+      <c r="R178" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S178" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T178" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U178" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V178" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W178" s="2" t="inlineStr"/>
+      <c r="X178" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y178" s="2" t="inlineStr">
+        <is>
+          <t>netzwerk</t>
+        </is>
+      </c>
+      <c r="Z178" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA178" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB178" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC178" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD178" s="2" t="inlineStr"/>
+      <c r="AE178" s="2" t="inlineStr"/>
+      <c r="AF178" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG178" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH178" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI178" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ178" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK178" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>J-00178</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Das Online-Banking der apoBank: neue Features</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Das Online-Banking der apoBank: neue Features</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr"/>
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/online-und-mobile-banking/neue-features</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L179" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M179" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N179" s="2" t="n"/>
+      <c r="O179" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P179" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q179" s="2" t="n"/>
+      <c r="R179" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S179" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T179" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U179" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V179" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W179" s="2" t="inlineStr"/>
+      <c r="X179" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y179" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z179" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA179" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB179" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC179" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD179" s="2" t="inlineStr"/>
+      <c r="AE179" s="2" t="inlineStr"/>
+      <c r="AF179" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG179" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH179" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI179" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ179" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK179" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>J-00179</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Banking Funktionen</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Banking Funktionen</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr"/>
+      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/online-und-mobile-banking/banking-funktionen</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L180" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M180" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N180" s="2" t="n"/>
+      <c r="O180" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P180" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q180" s="2" t="n"/>
+      <c r="R180" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S180" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T180" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U180" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V180" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W180" s="2" t="inlineStr"/>
+      <c r="X180" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y180" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z180" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA180" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB180" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC180" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD180" s="2" t="inlineStr"/>
+      <c r="AE180" s="2" t="inlineStr"/>
+      <c r="AF180" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG180" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH180" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI180" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ180" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK180" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>J-00180</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>Apps und Software</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Apps und Software</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr"/>
+      <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/online-und-mobile-banking/apps-und-software</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L181" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M181" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N181" s="2" t="n"/>
+      <c r="O181" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P181" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q181" s="2" t="n"/>
+      <c r="R181" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S181" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T181" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U181" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V181" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W181" s="2" t="inlineStr"/>
+      <c r="X181" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y181" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z181" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA181" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB181" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC181" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD181" s="2" t="inlineStr"/>
+      <c r="AE181" s="2" t="inlineStr"/>
+      <c r="AF181" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG181" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH181" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI181" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ181" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK181" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>J-00181</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Funktionen | apoBank-App</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Funktionen | apoBank-App</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr"/>
+      <c r="I182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/online-und-mobile-banking/apps-und-software/weiterleitung-apobank-app</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N182" s="2" t="n"/>
+      <c r="O182" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P182" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q182" s="2" t="n"/>
+      <c r="R182" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S182" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T182" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U182" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V182" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W182" s="2" t="inlineStr"/>
+      <c r="X182" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y182" s="2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="Z182" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA182" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB182" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC182" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD182" s="2" t="inlineStr"/>
+      <c r="AE182" s="2" t="inlineStr"/>
+      <c r="AF182" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG182" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH182" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI182" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ182" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK182" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>J-00182</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>FAQ | apoBank-App</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>FAQ | apoBank-App</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr"/>
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/online-und-mobile-banking/apps-und-software/faq-apobank-app</t>
+        </is>
+      </c>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L183" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M183" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N183" s="2" t="n"/>
+      <c r="O183" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P183" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q183" s="2" t="n"/>
+      <c r="R183" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S183" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T183" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U183" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V183" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W183" s="2" t="inlineStr"/>
+      <c r="X183" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y183" s="2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="Z183" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA183" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB183" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC183" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD183" s="2" t="inlineStr"/>
+      <c r="AE183" s="2" t="inlineStr"/>
+      <c r="AF183" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG183" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH183" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI183" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ183" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK183" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>J-00183</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Aktuelle Sicherheitshinweise</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>Aktuelle Sicherheitshinweise</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr"/>
+      <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/sicherheit/aktuelle-sicherheitshinweise</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L184" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="n"/>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P184" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q184" s="2" t="n"/>
+      <c r="R184" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S184" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T184" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U184" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V184" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W184" s="2" t="inlineStr"/>
+      <c r="X184" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y184" s="2" t="inlineStr">
+        <is>
+          <t>sicherheit</t>
+        </is>
+      </c>
+      <c r="Z184" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA184" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB184" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC184" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD184" s="2" t="inlineStr"/>
+      <c r="AE184" s="2" t="inlineStr"/>
+      <c r="AF184" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG184" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH184" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI184" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ184" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK184" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>J-00184</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>Sicherer Umgang im Online- und Mobile-Banking</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Sicherer Umgang im Online- und Mobile-Banking</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr"/>
+      <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/sicherheit/sicherer-umgang-im-online-und-mobile-banking</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N185" s="2" t="n"/>
+      <c r="O185" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P185" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q185" s="2" t="n"/>
+      <c r="R185" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S185" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T185" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U185" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V185" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W185" s="2" t="inlineStr"/>
+      <c r="X185" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y185" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z185" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA185" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB185" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC185" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD185" s="2" t="inlineStr"/>
+      <c r="AE185" s="2" t="inlineStr"/>
+      <c r="AF185" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG185" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH185" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI185" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ185" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK185" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>J-00185</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Unsere Sicherheitsverfahren</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Unsere Sicherheitsverfahren</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr"/>
+      <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/service/sicherheit/unsere-sicherheitsverfahren</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N186" s="2" t="n"/>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P186" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q186" s="2" t="n"/>
+      <c r="R186" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S186" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T186" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U186" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V186" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W186" s="2" t="inlineStr"/>
+      <c r="X186" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y186" s="2" t="inlineStr">
+        <is>
+          <t>sicherheit</t>
+        </is>
+      </c>
+      <c r="Z186" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA186" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB186" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC186" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD186" s="2" t="inlineStr"/>
+      <c r="AE186" s="2" t="inlineStr"/>
+      <c r="AF186" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG186" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH186" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI186" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ186" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK186" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>J-00186</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>Cookie-Einstellungen</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Cookie-Einstellungen</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr"/>
+      <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Apotheker- und Ärztebank eG - apoBank</t>
+        </is>
+      </c>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>deutscheapotherundärztebankapobank</t>
+        </is>
+      </c>
+      <c r="M187" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N187" s="2" t="n"/>
+      <c r="O187" s="2" t="inlineStr">
+        <is>
+          <t>Schloßplatz 6</t>
+        </is>
+      </c>
+      <c r="P187" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 2721164</t>
+        </is>
+      </c>
+      <c r="Q187" s="2" t="n"/>
+      <c r="R187" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S187" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T187" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de/studenten/karrierekompass-heilberufler</t>
+        </is>
+      </c>
+      <c r="U187" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apobank.de</t>
+        </is>
+      </c>
+      <c r="V187" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Deutsche Apotheker- und Ärztebank eG - apoBank_career.html</t>
+        </is>
+      </c>
+      <c r="W187" s="2" t="inlineStr"/>
+      <c r="X187" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y187" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z187" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA187" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB187" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC187" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD187" s="2" t="inlineStr"/>
+      <c r="AE187" s="2" t="inlineStr"/>
+      <c r="AF187" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AG187" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH187" s="2" t="n">
+        <v>2445</v>
+      </c>
+      <c r="AI187" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ187" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+      <c r="AK187" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25481,7 +29674,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>159</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2">
@@ -25492,7 +29685,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-14 15:35</t>
+          <t>2026-05-14 15:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Junior IT Jobs - 255 jobs (15:36)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
+++ b/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK242"/>
+  <dimension ref="A1:AK256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -37929,6 +37929,2266 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>J-00242</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Lage im Stadtplan</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>Lage im Stadtplan</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr"/>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>Untermenü
+Bildung und Wissenschaft
+Familie, Jugend und Soziales
+Gesundheit
+Planen, Bauen, Wohnen
+Verkehr und Infrastruktur
+Baustellen-Info
+Bahnausbau
+Fahrradstadt Bamberg
+Kommunale Wärmeplanung
+Verkehrsentwicklungsplan Bamberg
+Klima, Umwelt und Nachhaltigkeit
+ Vorlesen
+Inhalt
+Baustellen-Info
+Liebe Bürgerinnen und Bürger,
+mit unseren tagesaktuellen Informationen zu den Verkehrsbehinderungen durch Baustellen im Stadtgebiet sind Sie immer bestens informiert. Sie möchten die aktuellen Infos gern a</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/#gmc_anker</t>
+        </is>
+      </c>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L243" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M243" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N243" s="2" t="n"/>
+      <c r="O243" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P243" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q243" s="2" t="n"/>
+      <c r="R243" s="2" t="n"/>
+      <c r="S243" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T243" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U243" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V243" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W243" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Universität Erlangen-Nürnberg_ Lehrstuhl_Lage im Stadtplan.html</t>
+        </is>
+      </c>
+      <c r="X243" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y243" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="Z243" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA243" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB243" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC243" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD243" s="2" t="inlineStr"/>
+      <c r="AE243" s="2" t="inlineStr"/>
+      <c r="AF243" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG243" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH243" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI243" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ243" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK243" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>J-00243</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>nach oben</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>nach oben</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr"/>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>Untermenü
+Bildung und Wissenschaft
+Familie, Jugend und Soziales
+Gesundheit
+Planen, Bauen, Wohnen
+Verkehr und Infrastruktur
+Baustellen-Info
+Bahnausbau
+Fahrradstadt Bamberg
+Kommunale Wärmeplanung
+Verkehrsentwicklungsplan Bamberg
+Klima, Umwelt und Nachhaltigkeit
+ Vorlesen
+Inhalt
+Baustellen-Info
+Liebe Bürgerinnen und Bürger,
+mit unseren tagesaktuellen Informationen zu den Verkehrsbehinderungen durch Baustellen im Stadtgebiet sind Sie immer bestens informiert. Sie möchten die aktuellen Infos gern a</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/#top</t>
+        </is>
+      </c>
+      <c r="K244" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L244" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M244" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N244" s="2" t="n"/>
+      <c r="O244" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P244" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q244" s="2" t="n"/>
+      <c r="R244" s="2" t="n"/>
+      <c r="S244" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T244" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U244" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V244" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W244" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Universität Erlangen-Nürnberg_ Lehrstuhl_nach oben.html</t>
+        </is>
+      </c>
+      <c r="X244" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y244" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="Z244" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA244" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB244" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC244" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD244" s="2" t="inlineStr"/>
+      <c r="AE244" s="2" t="inlineStr"/>
+      <c r="AF244" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG244" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH244" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI244" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ244" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK244" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>J-00244</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg digital</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg digital</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr"/>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>Untermenü
+Bamberg digital
+Über uns
+Digitales Rathaus
+ Vorlesen
+Inhalt
+Bamberg digital
+Über uns
+Digitales Rathaus
+Themen
+© Stadt Bamberg, Smart City
+Smart City Bamberg
+Online Terminbuchung
+Bürgerbeteiligung der Stadt Bamberg
+BayernApp
+Weitere Informationen
+Adresse
+Stadtverwaltung Bamberg  •  Maximiliansplatz 3  •  96047 Bamberg  •   0951 87-0  •   0951 87-1964</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Bamberg-digital/</t>
+        </is>
+      </c>
+      <c r="K245" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L245" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M245" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N245" s="2" t="n"/>
+      <c r="O245" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P245" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q245" s="2" t="n"/>
+      <c r="R245" s="2" t="n"/>
+      <c r="S245" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T245" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U245" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V245" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W245" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Universität Erlangen-Nürnberg_ Lehrstuhl_Bamberg digital.html</t>
+        </is>
+      </c>
+      <c r="X245" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y245" s="2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="Z245" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA245" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB245" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC245" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD245" s="2" t="inlineStr"/>
+      <c r="AE245" s="2" t="inlineStr"/>
+      <c r="AF245" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG245" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH245" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI245" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ245" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK245" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>J-00245</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Digitales Rathaus</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>Digitales Rathaus</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>UX/UI Design</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>Vor Ort</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr"/>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>Untermenü
+Bamberg digital
+Über uns
+Digitales Rathaus
+ Vorlesen
+Inhalt
+Rund um die Uhr zu Ihrer Verwaltung
+"Auf dem Weg zu einem »Digitalen Rathaus« sind wir inzwischen wieder ein gutes Stück vorangekommen. So wurde die Stadt Bamberg jüngst als eine von sechs Städten in Bayern ausgezeichnet, die bereits über 50 Bürgerdienstleistungen online anbietet.
+Aber angesichts vieler verbleibender Dienstleistungen, für die noch kein digitales Verfahren zur Verfügung steht, müssen wir noch besser werden. I</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Bamberg-digital/Digitales-Rathaus/</t>
+        </is>
+      </c>
+      <c r="K246" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L246" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M246" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N246" s="2" t="n"/>
+      <c r="O246" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P246" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q246" s="2" t="n"/>
+      <c r="R246" s="2" t="n"/>
+      <c r="S246" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T246" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U246" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V246" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W246" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Universität Erlangen-Nürnberg_ Lehrstuhl_Digitales Rathaus.html</t>
+        </is>
+      </c>
+      <c r="X246" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y246" s="2" t="inlineStr">
+        <is>
+          <t>digitalisierung</t>
+        </is>
+      </c>
+      <c r="Z246" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA246" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB246" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC246" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD246" s="2" t="inlineStr"/>
+      <c r="AE246" s="2" t="inlineStr"/>
+      <c r="AF246" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG246" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH246" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI246" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ246" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK246" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>J-00246</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>KiTa-Portal</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>KiTa-Portal</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr"/>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>Untermenü
+Bildung und Wissenschaft
+Familie, Jugend und Soziales
+Asyl-Portal
+Ehrenamtskarte
+Familien
+Inklusion
+Jugend-Portal
+KiTa-Portal
+webKITA
+Menschen mit Behinderung
+Migrantinnen und Migranten
+Seniorinnen und Senioren
+Bamberger Bürgervereine
+Gesundheit
+Planen, Bauen, Wohnen
+Verkehr und Infrastruktur
+Klima, Umwelt und Nachhaltigkeit
+ Vorlesen
+Inhalt
+KiTa-Portal
+Sie sind alleinerziehend oder eine Familie mit Kindern? Die Stadt Bamberg verfügt über ein breitgefächertes Netz an Kindertagesstätte</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Familie-Jugend-und-Soziales/KiTa-Portal/</t>
+        </is>
+      </c>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L247" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M247" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N247" s="2" t="n"/>
+      <c r="O247" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P247" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q247" s="2" t="n"/>
+      <c r="R247" s="2" t="n"/>
+      <c r="S247" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T247" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U247" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V247" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W247" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/Universität Erlangen-Nürnberg_ Lehrstuhl_KiTa-Portal.html</t>
+        </is>
+      </c>
+      <c r="X247" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y247" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z247" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA247" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB247" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="AC247" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD247" s="2" t="inlineStr"/>
+      <c r="AE247" s="2" t="inlineStr"/>
+      <c r="AF247" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG247" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH247" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI247" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ247" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK247" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>J-00247</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Verkehr und Infrastruktur</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>Verkehr und Infrastruktur</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr"/>
+      <c r="I248" s="2" t="inlineStr"/>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/</t>
+        </is>
+      </c>
+      <c r="K248" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L248" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M248" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N248" s="2" t="n"/>
+      <c r="O248" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P248" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q248" s="2" t="n"/>
+      <c r="R248" s="2" t="n"/>
+      <c r="S248" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T248" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U248" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V248" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W248" s="2" t="inlineStr"/>
+      <c r="X248" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y248" s="2" t="inlineStr">
+        <is>
+          <t>infrastruktur</t>
+        </is>
+      </c>
+      <c r="Z248" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA248" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB248" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC248" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD248" s="2" t="inlineStr"/>
+      <c r="AE248" s="2" t="inlineStr"/>
+      <c r="AF248" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG248" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH248" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI248" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ248" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK248" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>J-00248</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Projekte und Aktionen</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>Projekte und Aktionen</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr"/>
+      <c r="I249" s="2" t="inlineStr"/>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Klima-Umwelt-und-Nachhaltigkeit/Nachhaltigkeit/Projekte-und-Aktionen/</t>
+        </is>
+      </c>
+      <c r="K249" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L249" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M249" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N249" s="2" t="n"/>
+      <c r="O249" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P249" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q249" s="2" t="n"/>
+      <c r="R249" s="2" t="n"/>
+      <c r="S249" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T249" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U249" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V249" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W249" s="2" t="inlineStr"/>
+      <c r="X249" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y249" s="2" t="inlineStr">
+        <is>
+          <t>projekt</t>
+        </is>
+      </c>
+      <c r="Z249" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA249" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB249" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC249" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD249" s="2" t="inlineStr"/>
+      <c r="AE249" s="2" t="inlineStr"/>
+      <c r="AF249" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG249" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH249" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI249" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ249" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK249" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>J-00249</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Klimaschutzprojekte</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>Klimaschutzprojekte</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr"/>
+      <c r="I250" s="2" t="inlineStr"/>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Klima-Umwelt-und-Nachhaltigkeit/Klimaschutzprojekte/</t>
+        </is>
+      </c>
+      <c r="K250" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L250" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M250" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N250" s="2" t="n"/>
+      <c r="O250" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P250" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q250" s="2" t="n"/>
+      <c r="R250" s="2" t="n"/>
+      <c r="S250" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T250" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U250" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V250" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W250" s="2" t="inlineStr"/>
+      <c r="X250" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y250" s="2" t="inlineStr">
+        <is>
+          <t>projekt</t>
+        </is>
+      </c>
+      <c r="Z250" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA250" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB250" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC250" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD250" s="2" t="inlineStr"/>
+      <c r="AE250" s="2" t="inlineStr"/>
+      <c r="AF250" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG250" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH250" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI250" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ250" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK250" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>J-00250</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>Film und Kino</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>Film und Kino</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="inlineStr"/>
+      <c r="I251" s="2" t="inlineStr"/>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Unsere-Stadt/Kultur-und-Kunst-/Film-und-Kino/</t>
+        </is>
+      </c>
+      <c r="K251" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L251" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M251" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N251" s="2" t="n"/>
+      <c r="O251" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P251" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q251" s="2" t="n"/>
+      <c r="R251" s="2" t="n"/>
+      <c r="S251" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T251" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U251" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V251" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W251" s="2" t="inlineStr"/>
+      <c r="X251" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y251" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z251" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA251" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB251" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC251" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD251" s="2" t="inlineStr"/>
+      <c r="AE251" s="2" t="inlineStr"/>
+      <c r="AF251" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG251" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH251" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI251" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ251" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK251" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>J-00251</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>Kinder- und Jugendkultur</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>Kinder- und Jugendkultur</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr"/>
+      <c r="I252" s="2" t="inlineStr"/>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Unsere-Stadt/Kultur-und-Kunst-/Kinder-und-Jugendkultur/</t>
+        </is>
+      </c>
+      <c r="K252" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L252" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M252" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N252" s="2" t="n"/>
+      <c r="O252" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P252" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q252" s="2" t="n"/>
+      <c r="R252" s="2" t="n"/>
+      <c r="S252" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T252" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U252" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V252" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W252" s="2" t="inlineStr"/>
+      <c r="X252" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y252" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z252" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA252" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB252" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC252" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD252" s="2" t="inlineStr"/>
+      <c r="AE252" s="2" t="inlineStr"/>
+      <c r="AF252" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG252" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH252" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI252" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ252" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK252" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>J-00252</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Feldkirchen</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>Feldkirchen</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="inlineStr"/>
+      <c r="I253" s="2" t="inlineStr"/>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Unsere-Stadt/Partnerst%C3%A4dte/Feldkirchen/</t>
+        </is>
+      </c>
+      <c r="K253" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L253" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M253" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N253" s="2" t="n"/>
+      <c r="O253" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P253" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q253" s="2" t="n"/>
+      <c r="R253" s="2" t="n"/>
+      <c r="S253" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T253" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U253" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V253" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W253" s="2" t="inlineStr"/>
+      <c r="X253" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y253" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z253" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA253" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB253" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC253" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD253" s="2" t="inlineStr"/>
+      <c r="AE253" s="2" t="inlineStr"/>
+      <c r="AF253" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG253" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH253" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI253" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ253" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK253" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>J-00253</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Informationstechnologie</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>Informationstechnologie</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr"/>
+      <c r="I254" s="2" t="inlineStr"/>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Wirtschaft/Fokusbranchen/Informationstechnologie/</t>
+        </is>
+      </c>
+      <c r="K254" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L254" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M254" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N254" s="2" t="n"/>
+      <c r="O254" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P254" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q254" s="2" t="n"/>
+      <c r="R254" s="2" t="n"/>
+      <c r="S254" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T254" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U254" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V254" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W254" s="2" t="inlineStr"/>
+      <c r="X254" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y254" s="2" t="inlineStr">
+        <is>
+          <t>technologie</t>
+        </is>
+      </c>
+      <c r="Z254" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA254" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB254" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC254" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD254" s="2" t="inlineStr"/>
+      <c r="AE254" s="2" t="inlineStr"/>
+      <c r="AF254" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG254" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH254" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI254" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ254" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK254" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>J-00254</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg: a focal point in the network of Metropolitan Regions</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg: a focal point in the network of Metropolitan Regions</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr"/>
+      <c r="I255" s="2" t="inlineStr"/>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Wirtschaft/English-Pages/Bamberg-a-focal-point-in-the-network-of-Metropolitan-Regions/</t>
+        </is>
+      </c>
+      <c r="K255" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L255" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M255" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N255" s="2" t="n"/>
+      <c r="O255" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P255" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q255" s="2" t="n"/>
+      <c r="R255" s="2" t="n"/>
+      <c r="S255" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T255" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U255" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V255" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W255" s="2" t="inlineStr"/>
+      <c r="X255" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y255" s="2" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="Z255" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA255" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB255" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC255" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD255" s="2" t="inlineStr"/>
+      <c r="AE255" s="2" t="inlineStr"/>
+      <c r="AF255" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG255" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH255" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI255" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ255" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK255" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>J-00255</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>E-Mail:sicheres Kontaktformular</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>E-Mail:sicheres Kontaktformular</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr"/>
+      <c r="I256" s="2" t="inlineStr"/>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>https://formularserver-bp.bayern.de/sichererKontakt?caller=23109316387</t>
+        </is>
+      </c>
+      <c r="K256" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg: Lehrstuhl für Kunststofftechnik</t>
+        </is>
+      </c>
+      <c r="L256" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberglehrstuhlfürkunststofftechnik</t>
+        </is>
+      </c>
+      <c r="M256" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N256" s="2" t="n"/>
+      <c r="O256" s="2" t="inlineStr">
+        <is>
+          <t>Weichselgarten 10</t>
+        </is>
+      </c>
+      <c r="P256" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8571000</t>
+        </is>
+      </c>
+      <c r="Q256" s="2" t="n"/>
+      <c r="R256" s="2" t="n"/>
+      <c r="S256" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T256" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/Leben/Verkehr-und-Infrastruktur/Baustellen-Info/</t>
+        </is>
+      </c>
+      <c r="U256" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadt.bamberg.de/B%C3%BCrgerservice/Beh%C3%B6rdenwegweiser/Technisches-Rathaus/index.php?object=tx,3481.1&amp;ModID=9&amp;FID=1829.328.1&amp;NavID=3481.1783&amp;La=1</t>
+        </is>
+      </c>
+      <c r="V256" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg_ Lehrstuhl für Kunststofftechnik_career.html</t>
+        </is>
+      </c>
+      <c r="W256" s="2" t="inlineStr"/>
+      <c r="X256" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y256" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z256" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA256" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB256" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC256" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD256" s="2" t="inlineStr"/>
+      <c r="AE256" s="2" t="inlineStr"/>
+      <c r="AF256" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AG256" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH256" s="2" t="n">
+        <v>2377</v>
+      </c>
+      <c r="AI256" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ256" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+      <c r="AK256" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -37950,7 +40210,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>241</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Junior IT Jobs - 265 jobs (15:36)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
+++ b/download/Junior_IT_Jobs_Bamberg_Erlangen_Nuernberg.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK256"/>
+  <dimension ref="A1:AK266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -40189,6 +40189,1643 @@
         </is>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>J-00256</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Cookie-Informationen</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>Cookie-Informationen</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr"/>
+      <c r="I257" s="2" t="inlineStr"/>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>https://www.unifleisch.de/de/news-details/de/stellenangebote/</t>
+        </is>
+      </c>
+      <c r="K257" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg Geschäftsstelle Maschinenbau</t>
+        </is>
+      </c>
+      <c r="L257" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberggeschäftsstellemaschinenbau</t>
+        </is>
+      </c>
+      <c r="M257" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N257" s="2" t="n"/>
+      <c r="O257" s="2" t="inlineStr">
+        <is>
+          <t>Immerwahrstraße 2a</t>
+        </is>
+      </c>
+      <c r="P257" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8528769</t>
+        </is>
+      </c>
+      <c r="Q257" s="2" t="n"/>
+      <c r="R257" s="2" t="n"/>
+      <c r="S257" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T257" s="2" t="inlineStr">
+        <is>
+          <t>https://www.unifleisch.de/de/news-details/de/stellenangebote/</t>
+        </is>
+      </c>
+      <c r="U257" s="2" t="inlineStr">
+        <is>
+          <t>https://www.unifleisch.de/de/news-details/die-unifleisch-gruppe-uebernimmt-den-erlanger-schlachthof</t>
+        </is>
+      </c>
+      <c r="V257" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg Geschäftsstelle Maschinenbau_career.html</t>
+        </is>
+      </c>
+      <c r="W257" s="2" t="inlineStr"/>
+      <c r="X257" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y257" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z257" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA257" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB257" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC257" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD257" s="2" t="inlineStr"/>
+      <c r="AE257" s="2" t="inlineStr"/>
+      <c r="AF257" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG257" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH257" s="2" t="n">
+        <v>2584</v>
+      </c>
+      <c r="AI257" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ257" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK257" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>J-00257</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.myfonts.com/legal/website-use-privacy-policy</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.myfonts.com/legal/website-use-privacy-policy</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr"/>
+      <c r="I258" s="2" t="inlineStr"/>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.myfonts.com/legal/website-use-privacy-policy</t>
+        </is>
+      </c>
+      <c r="K258" s="2" t="inlineStr">
+        <is>
+          <t>Universität Erlangen-Nürnberg Geschäftsstelle Maschinenbau</t>
+        </is>
+      </c>
+      <c r="L258" s="2" t="inlineStr">
+        <is>
+          <t>universitäterlangennürnberggeschäftsstellemaschinenbau</t>
+        </is>
+      </c>
+      <c r="M258" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="N258" s="2" t="n"/>
+      <c r="O258" s="2" t="inlineStr">
+        <is>
+          <t>Immerwahrstraße 2a</t>
+        </is>
+      </c>
+      <c r="P258" s="2" t="inlineStr">
+        <is>
+          <t>+49 9131 8528769</t>
+        </is>
+      </c>
+      <c r="Q258" s="2" t="n"/>
+      <c r="R258" s="2" t="n"/>
+      <c r="S258" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.unifleisch.de/de/news-details/de/stellenangebote/</t>
+        </is>
+      </c>
+      <c r="U258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.unifleisch.de/de/news-details/die-unifleisch-gruppe-uebernimmt-den-erlanger-schlachthof</t>
+        </is>
+      </c>
+      <c r="V258" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/Universität Erlangen-Nürnberg Geschäftsstelle Maschinenbau_career.html</t>
+        </is>
+      </c>
+      <c r="W258" s="2" t="inlineStr"/>
+      <c r="X258" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y258" s="2" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Z258" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA258" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB258" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC258" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD258" s="2" t="inlineStr"/>
+      <c r="AE258" s="2" t="inlineStr"/>
+      <c r="AF258" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG258" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH258" s="2" t="n">
+        <v>2584</v>
+      </c>
+      <c r="AI258" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ258" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK258" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>J-00258</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>ZU DEN OFFENEN STELLEN</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>ZU DEN OFFENEN STELLEN</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t>java, angular, react, spring</t>
+        </is>
+      </c>
+      <c r="I259" s="2" t="inlineStr">
+        <is>
+          <t>Auf der Suche nach einer neuen Herausforderung?
+Offene Stellen
+Festanstellung (Bereich Tech)
+- 4 Positionen
+4
+Backend Developer KI (Associate Consultant Niveau) (m/w/d)
+Nürnberg
+Vollzeit
+Festanstellung
+Data Engineer (m/w/d)
+Nürnberg
+Vollzeit
+Festanstellung
+Fullstack Developer (m/w/d)
+Nürnberg
+Vollzeit
+Festanstellung
+Senior Fullstack Developer - Java EE/Spring/Angular/React (m/w/d)
+Nürnberg
+Vollzeit
+Festanstellung</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>https://codecampn.jobs.personio.de/</t>
+        </is>
+      </c>
+      <c r="K259" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L259" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M259" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N259" s="2" t="n"/>
+      <c r="O259" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P259" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q259" s="2" t="n"/>
+      <c r="R259" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S259" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T259" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U259" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V259" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W259" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/CodeCamp_N_ZU DEN OFFENEN STELLEN.html</t>
+        </is>
+      </c>
+      <c r="X259" s="2" t="inlineStr">
+        <is>
+          <t>associate</t>
+        </is>
+      </c>
+      <c r="Y259" s="2" t="inlineStr">
+        <is>
+          <t>developer</t>
+        </is>
+      </c>
+      <c r="Z259" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA259" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB259" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC259" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD259" s="2" t="inlineStr"/>
+      <c r="AE259" s="2" t="inlineStr"/>
+      <c r="AF259" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG259" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH259" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI259" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ259" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK259" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>J-00259</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>Mail schreiben</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>Mail schreiben</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr"/>
+      <c r="I260" s="2" t="inlineStr"/>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>mailto:elisabeth.krueger@codecamp-n.com?subject=Anfrage%20zur%20Bewerbung%20bei%20CodeCamp%3AN</t>
+        </is>
+      </c>
+      <c r="K260" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L260" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M260" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N260" s="2" t="n"/>
+      <c r="O260" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P260" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q260" s="2" t="n"/>
+      <c r="R260" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S260" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T260" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U260" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V260" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W260" s="2" t="inlineStr"/>
+      <c r="X260" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y260" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z260" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA260" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB260" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC260" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD260" s="2" t="inlineStr"/>
+      <c r="AE260" s="2" t="inlineStr"/>
+      <c r="AF260" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG260" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH260" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI260" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ260" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK260" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>J-00260</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr"/>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>選擇語言
+Bahasa Indonesia (Bahasa Indonesia)
+Bahasa Malaysia (Malay)
+Čeština (Czech)
+Dansk (Danish)
+Deutsch (German)
+English (English)
+Español (Spanish)
+繁體中文 (Chinese (Traditional))
+Français (French)
+한국어 (Korean)
+Italiano (Italian)
+简体中文 (Chinese (Simplified))
+Nederlands (Dutch)
+日本語 (Japanese)
+Norsk (Norwegian)
+Polski (Polish)
+Português (Portuguese)
+Română (Romanian)
+Русский (Russian)
+Svenska (Swedish)
+Tagalog (Tagalog)
+ภาษาไทย (Thai)
+Türkçe (Turkish)
+العربية (Arabic)
+Seite nicht gefunden
+Die gewünsc</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/elisabeth-kr%C3%BCger-51231b1ab/</t>
+        </is>
+      </c>
+      <c r="K261" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L261" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M261" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N261" s="2" t="n"/>
+      <c r="O261" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P261" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q261" s="2" t="n"/>
+      <c r="R261" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S261" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T261" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U261" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V261" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W261" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/CodeCamp_N_LinkedIn.html</t>
+        </is>
+      </c>
+      <c r="X261" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y261" s="2" t="inlineStr">
+        <is>
+          <t>netzwerk</t>
+        </is>
+      </c>
+      <c r="Z261" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA261" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB261" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC261" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD261" s="2" t="inlineStr"/>
+      <c r="AE261" s="2" t="inlineStr"/>
+      <c r="AF261" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG261" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH261" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI261" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ261" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK261" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>J-00261</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>Modernisierung IT-Landschaft</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>Modernisierung IT-Landschaft</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>devops</t>
+        </is>
+      </c>
+      <c r="I262" s="2" t="inlineStr">
+        <is>
+          <t>LEISTUNGEN
+BRANCHEN
+BLOG
+KARRIERE
+ÜBER UNS
+KONTAKT
+HOME
+LEISTUNGEN
+MODERNISIERUNG IT-LANDSCHAFT
+IT-Systeme und Software zukunftssicher machen
+BERATUNGSGESPRÄCH ANFRAGEN
+Auszug unserer Kund:innen und Partner:innen
+Herausforderungen gewachsener IT-Strukturen meistern
+Wir helfen Dir, Deine Software und IT-Systeme zukunftssicher zu machen, die Performance zu steigern und Kosten zu senken. Unser erfahrenes Team analysiert Deine aktuelle IT-Landschaft, identifiziert Optimierungspotenziale und entwick</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/leistungen/modernisierung-it-landschaft</t>
+        </is>
+      </c>
+      <c r="K262" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L262" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M262" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N262" s="2" t="n"/>
+      <c r="O262" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P262" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q262" s="2" t="n"/>
+      <c r="R262" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S262" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T262" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U262" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V262" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W262" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/junior_jobs_html/CodeCamp_N_Modernisierung IT-Landschaft.html</t>
+        </is>
+      </c>
+      <c r="X262" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y262" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z262" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA262" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB262" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC262" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD262" s="2" t="inlineStr"/>
+      <c r="AE262" s="2" t="inlineStr"/>
+      <c r="AF262" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG262" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH262" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI262" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ262" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK262" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>J-00262</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Softwarequalität</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>Softwarequalität</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr"/>
+      <c r="I263" s="2" t="inlineStr"/>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/leistungen/steigerung-softwarequalitat</t>
+        </is>
+      </c>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L263" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M263" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N263" s="2" t="n"/>
+      <c r="O263" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P263" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q263" s="2" t="n"/>
+      <c r="R263" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S263" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T263" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U263" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V263" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W263" s="2" t="inlineStr"/>
+      <c r="X263" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y263" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z263" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA263" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB263" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC263" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD263" s="2" t="inlineStr"/>
+      <c r="AE263" s="2" t="inlineStr"/>
+      <c r="AF263" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG263" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH263" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI263" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ263" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK263" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>J-00263</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Projektreferenzen</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Projektreferenzen</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr"/>
+      <c r="I264" s="2" t="inlineStr"/>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/projektreferenzen</t>
+        </is>
+      </c>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L264" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M264" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N264" s="2" t="n"/>
+      <c r="O264" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P264" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q264" s="2" t="n"/>
+      <c r="R264" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S264" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T264" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U264" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V264" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W264" s="2" t="inlineStr"/>
+      <c r="X264" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y264" s="2" t="inlineStr">
+        <is>
+          <t>projekt</t>
+        </is>
+      </c>
+      <c r="Z264" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA264" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB264" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC264" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD264" s="2" t="inlineStr"/>
+      <c r="AE264" s="2" t="inlineStr"/>
+      <c r="AF264" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG264" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH264" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI264" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ264" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK264" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>J-00264</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Erlebe Codecamp:NKlicke hier, um die 360-Grad-Tour zu starten.</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>Erlebe Codecamp:NKlicke hier, um die 360-Grad-Tour zu starten.</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr"/>
+      <c r="I265" s="2" t="inlineStr"/>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/360-grad-tour</t>
+        </is>
+      </c>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L265" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M265" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N265" s="2" t="n"/>
+      <c r="O265" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P265" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q265" s="2" t="n"/>
+      <c r="R265" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S265" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T265" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U265" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V265" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W265" s="2" t="inlineStr"/>
+      <c r="X265" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y265" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="Z265" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA265" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB265" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC265" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD265" s="2" t="inlineStr"/>
+      <c r="AE265" s="2" t="inlineStr"/>
+      <c r="AF265" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG265" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH265" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI265" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ265" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK265" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>J-00265</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>info@codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>info@codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr"/>
+      <c r="I266" s="2" t="inlineStr"/>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>mailto:info@codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>CodeCamp:N</t>
+        </is>
+      </c>
+      <c r="L266" s="2" t="inlineStr">
+        <is>
+          <t>codecampn</t>
+        </is>
+      </c>
+      <c r="M266" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberg</t>
+        </is>
+      </c>
+      <c r="N266" s="2" t="n"/>
+      <c r="O266" s="2" t="inlineStr">
+        <is>
+          <t>Solgerstraße 18</t>
+        </is>
+      </c>
+      <c r="P266" s="2" t="inlineStr">
+        <is>
+          <t>+49 911 27448523</t>
+        </is>
+      </c>
+      <c r="Q266" s="2" t="n"/>
+      <c r="R266" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="S266" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T266" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com/karriere</t>
+        </is>
+      </c>
+      <c r="U266" s="2" t="inlineStr">
+        <is>
+          <t>https://www.codecamp-n.com</t>
+        </is>
+      </c>
+      <c r="V266" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_html/CodeCamp_N_career.html</t>
+        </is>
+      </c>
+      <c r="W266" s="2" t="inlineStr"/>
+      <c r="X266" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y266" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="Z266" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA266" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB266" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="AC266" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="AD266" s="2" t="inlineStr"/>
+      <c r="AE266" s="2" t="inlineStr"/>
+      <c r="AF266" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AG266" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AH266" s="2" t="n">
+        <v>2382</v>
+      </c>
+      <c r="AI266" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="AJ266" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+      <c r="AK266" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 15:36:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -40210,7 +41847,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>255</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2">

</xml_diff>